<commit_message>
docs(schedule): «동승» 을 매뉴얼 2.3 · 교육 자료 1.5 · TC 185행 · CLAUDE.md 에 반영
- 매뉴얼 8.6 「차량이 겹칠 때 · 함께 탈 때」 — 셋 중 고르는 창 · 대표 · 동승 풀기 · 메일 제목
- 교육 자료 5.2 같은 내용 요약
- TC +11 (적합 177 · 미수행 8) — 테스트 서버(:8092)에서 화면으로 눌러 확인한 것만
  함께 타기 창 · 경고 사라짐 · 대표 판정 · 묶음 밖 겹침 · 창의 함께 타기 · 동승 풀기 ·
  날짜 변경 시 해제 · 배차표/일 보기 표시 · 메일 제목 · 차량 거리 한 번만(760→860) ·
  하이패스 후보 대표 1명
- CLAUDE.md 일정 관리에 «동승» 절 · 마이그 039 두 DB 적용 기록
- 겹침 창 설명의 「따로 등록」 → 「따로」 — 붙여넣기 단추는 「따로 붙이기」 라 문구가 어긋났다

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/testcase/TC_업무_현황_대시보드.xlsx
+++ b/docs/testcase/TC_업무_현황_대시보드.xlsx
@@ -756,7 +756,7 @@
     <row r="15" ht="24" customHeight="1">
       <c r="A15" s="7" t="inlineStr">
         <is>
-          <t>적합 166건 · 미수행 8건 · 부적합 0건</t>
+          <t>적합 177건 · 미수행 8건 · 부적합 0건</t>
         </is>
       </c>
       <c r="B15" s="5" t="n"/>
@@ -789,7 +789,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I177"/>
+  <dimension ref="A1:I188"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -7975,300 +7975,773 @@
         </is>
       </c>
     </row>
-    <row r="169" ht="20" customHeight="1">
-      <c r="A169" s="9" t="inlineStr">
+    <row r="169">
+      <c r="A169" s="10" t="inlineStr">
+        <is>
+          <t>TC-D-167</t>
+        </is>
+      </c>
+      <c r="B169" s="10" t="inlineStr">
+        <is>
+          <t>일정</t>
+        </is>
+      </c>
+      <c r="C169" s="4" t="inlineStr">
+        <is>
+          <t>같은 차를 이미 잡은 날 등록하면 «함께 타기·따로·취소» 를 묻는가?</t>
+        </is>
+      </c>
+      <c r="D169" s="4" t="inlineStr">
+        <is>
+          <t>윤인철이 잡은 차를 이건호 칸에 붙여 넣어 뜨는 창 확인</t>
+        </is>
+      </c>
+      <c r="E169" s="11" t="inlineStr">
+        <is>
+          <t>적합</t>
+        </is>
+      </c>
+      <c r="F169" s="10" t="inlineStr">
+        <is>
+          <t>이건호</t>
+        </is>
+      </c>
+      <c r="G169" s="10" t="inlineStr"/>
+      <c r="H169" s="4" t="inlineStr">
+        <is>
+          <t>「그래도 등록?」 만 뜨면 배포본이 옛것인지 확인</t>
+        </is>
+      </c>
+      <c r="I169" s="4" t="inlineStr">
+        <is>
+          <t>9/23 Model Y — 창에 「윤인철」 과 세 단추</t>
+        </is>
+      </c>
+    </row>
+    <row r="170">
+      <c r="A170" s="12" t="inlineStr">
+        <is>
+          <t>TC-D-168</t>
+        </is>
+      </c>
+      <c r="B170" s="12" t="inlineStr">
+        <is>
+          <t>일정</t>
+        </is>
+      </c>
+      <c r="C170" s="13" t="inlineStr">
+        <is>
+          <t>[함께 타기] 를 누르면 겹침 경고가 사라지는가?</t>
+        </is>
+      </c>
+      <c r="D170" s="13" t="inlineStr">
+        <is>
+          <t>함께 타기 뒤 달력 위 경고와 두 계획의 묶음 번호 확인</t>
+        </is>
+      </c>
+      <c r="E170" s="14" t="inlineStr">
+        <is>
+          <t>적합</t>
+        </is>
+      </c>
+      <c r="F170" s="12" t="inlineStr">
+        <is>
+          <t>이건호</t>
+        </is>
+      </c>
+      <c r="G170" s="12" t="inlineStr"/>
+      <c r="H170" s="13" t="inlineStr">
+        <is>
+          <t>경고가 남으면 겹침을 «배차 단위» 로 세는지 확인</t>
+        </is>
+      </c>
+      <c r="I170" s="13" t="inlineStr">
+        <is>
+          <t>묶음 238 · 경고 없음 · 두 배지에 👥</t>
+        </is>
+      </c>
+    </row>
+    <row r="171">
+      <c r="A171" s="10" t="inlineStr">
+        <is>
+          <t>TC-D-169</t>
+        </is>
+      </c>
+      <c r="B171" s="10" t="inlineStr">
+        <is>
+          <t>일정</t>
+        </is>
+      </c>
+      <c r="C171" s="4" t="inlineStr">
+        <is>
+          <t>먼저 잡은 사람이 대표가 되는가?</t>
+        </is>
+      </c>
+      <c r="D171" s="4" t="inlineStr">
+        <is>
+          <t>두 계획의 동승자 여부(carpool_rider) 확인</t>
+        </is>
+      </c>
+      <c r="E171" s="11" t="inlineStr">
+        <is>
+          <t>적합</t>
+        </is>
+      </c>
+      <c r="F171" s="10" t="inlineStr">
+        <is>
+          <t>이건호</t>
+        </is>
+      </c>
+      <c r="G171" s="10" t="inlineStr"/>
+      <c r="H171" s="4" t="inlineStr">
+        <is>
+          <t>뒤 사람이 대표면 번호 순서 판정 확인</t>
+        </is>
+      </c>
+      <c r="I171" s="4" t="inlineStr">
+        <is>
+          <t>238 윤인철(먼저) 대표 · 239 이건호 동승</t>
+        </is>
+      </c>
+    </row>
+    <row r="172">
+      <c r="A172" s="12" t="inlineStr">
+        <is>
+          <t>TC-D-170</t>
+        </is>
+      </c>
+      <c r="B172" s="12" t="inlineStr">
+        <is>
+          <t>일정</t>
+        </is>
+      </c>
+      <c r="C172" s="13" t="inlineStr">
+        <is>
+          <t>묶음 밖의 사람이 따로 잡으면 다시 겹침으로 보이는가?</t>
+        </is>
+      </c>
+      <c r="D172" s="13" t="inlineStr">
+        <is>
+          <t>세 번째 사람을 «따로» 등록해 경고 확인</t>
+        </is>
+      </c>
+      <c r="E172" s="14" t="inlineStr">
+        <is>
+          <t>적합</t>
+        </is>
+      </c>
+      <c r="F172" s="12" t="inlineStr">
+        <is>
+          <t>이건호</t>
+        </is>
+      </c>
+      <c r="G172" s="12" t="inlineStr"/>
+      <c r="H172" s="13" t="inlineStr">
+        <is>
+          <t>안 뜨면 묶음 밖 계획까지 빼고 있는지 확인</t>
+        </is>
+      </c>
+      <c r="I172" s="13" t="inlineStr">
+        <is>
+          <t>「윤인철 · 이건호 · 김동현」 경고 — 배차 단위 둘</t>
+        </is>
+      </c>
+    </row>
+    <row r="173">
+      <c r="A173" s="10" t="inlineStr">
+        <is>
+          <t>TC-D-171</t>
+        </is>
+      </c>
+      <c r="B173" s="10" t="inlineStr">
+        <is>
+          <t>일정</t>
+        </is>
+      </c>
+      <c r="C173" s="4" t="inlineStr">
+        <is>
+          <t>이미 넣은 계획을 창에서 [함께 타기] 로 묶을 수 있는가?</t>
+        </is>
+      </c>
+      <c r="D173" s="4" t="inlineStr">
+        <is>
+          <t>겹친 사람의 계획 창 붉은 상자에서 [👥 함께 타기] 누르기</t>
+        </is>
+      </c>
+      <c r="E173" s="11" t="inlineStr">
+        <is>
+          <t>적합</t>
+        </is>
+      </c>
+      <c r="F173" s="10" t="inlineStr">
+        <is>
+          <t>이건호</t>
+        </is>
+      </c>
+      <c r="G173" s="10" t="inlineStr"/>
+      <c r="H173" s="4" t="inlineStr">
+        <is>
+          <t>단추가 없으면 겹친 상대가 한 묶음인지 확인</t>
+        </is>
+      </c>
+      <c r="I173" s="4" t="inlineStr">
+        <is>
+          <t>김동현 → 세 명 묶음 · 경고 사라짐</t>
+        </is>
+      </c>
+    </row>
+    <row r="174">
+      <c r="A174" s="12" t="inlineStr">
+        <is>
+          <t>TC-D-172</t>
+        </is>
+      </c>
+      <c r="B174" s="12" t="inlineStr">
+        <is>
+          <t>일정</t>
+        </is>
+      </c>
+      <c r="C174" s="13" t="inlineStr">
+        <is>
+          <t>[동승 풀기] 가 «그 사람만» 빼는가?</t>
+        </is>
+      </c>
+      <c r="D174" s="13" t="inlineStr">
+        <is>
+          <t>동승자 창의 [동승 풀기] 뒤 남은 묶음과 경고 확인</t>
+        </is>
+      </c>
+      <c r="E174" s="14" t="inlineStr">
+        <is>
+          <t>적합</t>
+        </is>
+      </c>
+      <c r="F174" s="12" t="inlineStr">
+        <is>
+          <t>이건호</t>
+        </is>
+      </c>
+      <c r="G174" s="12" t="inlineStr"/>
+      <c r="H174" s="13" t="inlineStr">
+        <is>
+          <t>묶음 전체가 풀리면 풀기 대상 조건 확인</t>
+        </is>
+      </c>
+      <c r="I174" s="13" t="inlineStr">
+        <is>
+          <t>이건호만 빠짐 · 윤인철+김동현 유지 · 경고 다시 뜸</t>
+        </is>
+      </c>
+    </row>
+    <row r="175">
+      <c r="A175" s="10" t="inlineStr">
+        <is>
+          <t>TC-D-173</t>
+        </is>
+      </c>
+      <c r="B175" s="10" t="inlineStr">
+        <is>
+          <t>일정</t>
+        </is>
+      </c>
+      <c r="C175" s="4" t="inlineStr">
+        <is>
+          <t>날짜를 바꾸면 동승에서 저절로 빠지는가?</t>
+        </is>
+      </c>
+      <c r="D175" s="4" t="inlineStr">
+        <is>
+          <t>동승 계획의 날짜를 하루 옮긴 뒤 묶음 번호 확인</t>
+        </is>
+      </c>
+      <c r="E175" s="11" t="inlineStr">
+        <is>
+          <t>적합</t>
+        </is>
+      </c>
+      <c r="F175" s="10" t="inlineStr">
+        <is>
+          <t>이건호</t>
+        </is>
+      </c>
+      <c r="G175" s="10" t="inlineStr"/>
+      <c r="H175" s="4" t="inlineStr">
+        <is>
+          <t>남으면 다른 날 예약이 겹침 검사에서 조용히 빠진다</t>
+        </is>
+      </c>
+      <c r="I175" s="4" t="inlineStr">
+        <is>
+          <t>9/23 → 9/22 · 묶음 번호 비워짐</t>
+        </is>
+      </c>
+    </row>
+    <row r="176">
+      <c r="A176" s="12" t="inlineStr">
+        <is>
+          <t>TC-D-174</t>
+        </is>
+      </c>
+      <c r="B176" s="12" t="inlineStr">
+        <is>
+          <t>화면</t>
+        </is>
+      </c>
+      <c r="C176" s="13" t="inlineStr">
+        <is>
+          <t>배차표·일 보기에서 동승이 겹침 대신 «동승» 으로 보이는가?</t>
+        </is>
+      </c>
+      <c r="D176" s="13" t="inlineStr">
+        <is>
+          <t>차량 기준 주 보기와 일 보기 「차량 배정」 확인</t>
+        </is>
+      </c>
+      <c r="E176" s="14" t="inlineStr">
+        <is>
+          <t>적합</t>
+        </is>
+      </c>
+      <c r="F176" s="12" t="inlineStr">
+        <is>
+          <t>이건호</t>
+        </is>
+      </c>
+      <c r="G176" s="12" t="inlineStr"/>
+      <c r="H176" s="13" t="inlineStr">
+        <is>
+          <t>「겹침」 이 뜨면 공용 달력 조각이 배차 단위를 세는지 확인</t>
+        </is>
+      </c>
+      <c r="I176" s="13" t="inlineStr">
+        <is>
+          <t>「👥 동승 3명」 · 일 보기 대표 1 · 동승 2 · 겹침 없음</t>
+        </is>
+      </c>
+    </row>
+    <row r="177">
+      <c r="A177" s="10" t="inlineStr">
+        <is>
+          <t>TC-D-175</t>
+        </is>
+      </c>
+      <c r="B177" s="10" t="inlineStr">
+        <is>
+          <t>메일</t>
+        </is>
+      </c>
+      <c r="C177" s="4" t="inlineStr">
+        <is>
+          <t>함께 타기 메일 제목에 「동승」 이 붙는가?</t>
+        </is>
+      </c>
+      <c r="D177" s="4" t="inlineStr">
+        <is>
+          <t>함께 타기 뒤 서버 발송 기록 확인</t>
+        </is>
+      </c>
+      <c r="E177" s="11" t="inlineStr">
+        <is>
+          <t>적합</t>
+        </is>
+      </c>
+      <c r="F177" s="10" t="inlineStr">
+        <is>
+          <t>이건호</t>
+        </is>
+      </c>
+      <c r="G177" s="10" t="inlineStr"/>
+      <c r="H177" s="4" t="inlineStr">
+        <is>
+          <t>「등록」 으로 가면 동승자 판정을 확인</t>
+        </is>
+      </c>
+      <c r="I177" s="4" t="inlineStr">
+        <is>
+          <t>「[차량] 동승 · 이건호 · 9/23(수) · Model Y 15도 3955 · 함께: 윤인철」 — 시험 주소로</t>
+        </is>
+      </c>
+    </row>
+    <row r="178">
+      <c r="A178" s="12" t="inlineStr">
+        <is>
+          <t>TC-D-176</t>
+        </is>
+      </c>
+      <c r="B178" s="12" t="inlineStr">
+        <is>
+          <t>정산</t>
+        </is>
+      </c>
+      <c r="C178" s="13" t="inlineStr">
+        <is>
+          <t>동승자의 실적이 차량 주행거리에 «두 번» 세어지지 않는가?</t>
+        </is>
+      </c>
+      <c r="D178" s="13" t="inlineStr">
+        <is>
+          <t>지난 날짜에 동승 2건(각 100km) 실적을 넣고 차량별 주행거리 확인</t>
+        </is>
+      </c>
+      <c r="E178" s="14" t="inlineStr">
+        <is>
+          <t>적합</t>
+        </is>
+      </c>
+      <c r="F178" s="12" t="inlineStr">
+        <is>
+          <t>이건호</t>
+        </is>
+      </c>
+      <c r="G178" s="12" t="inlineStr"/>
+      <c r="H178" s="13" t="inlineStr">
+        <is>
+          <t>200 늘면 차량별 합계에서 동승자를 빼는지 확인</t>
+        </is>
+      </c>
+      <c r="I178" s="13" t="inlineStr">
+        <is>
+          <t>Model Y 760 → 860km(한 번만) · 두 사람 업무 거리는 각각 +100km · 지운 뒤 760 복귀</t>
+        </is>
+      </c>
+    </row>
+    <row r="179">
+      <c r="A179" s="10" t="inlineStr">
+        <is>
+          <t>TC-D-177</t>
+        </is>
+      </c>
+      <c r="B179" s="10" t="inlineStr">
+        <is>
+          <t>하이패스</t>
+        </is>
+      </c>
+      <c r="C179" s="4" t="inlineStr">
+        <is>
+          <t>동승한 날 통행의 후보가 «대표 한 명» 인가?</t>
+        </is>
+      </c>
+      <c r="D179" s="4" t="inlineStr">
+        <is>
+          <t>그날 그 차에 수기 통행을 넣고 후보 목록 확인</t>
+        </is>
+      </c>
+      <c r="E179" s="11" t="inlineStr">
+        <is>
+          <t>적합</t>
+        </is>
+      </c>
+      <c r="F179" s="10" t="inlineStr">
+        <is>
+          <t>이건호</t>
+        </is>
+      </c>
+      <c r="G179" s="10" t="inlineStr"/>
+      <c r="H179" s="4" t="inlineStr">
+        <is>
+          <t>둘이 나오면 후보 조회가 동승자를 빼는지 확인</t>
+        </is>
+      </c>
+      <c r="I179" s="4" t="inlineStr">
+        <is>
+          <t>후보 윤인철 1명 — 자동 배정이 「애매」 로 남지 않는다</t>
+        </is>
+      </c>
+    </row>
+    <row r="180" ht="20" customHeight="1">
+      <c r="A180" s="9" t="inlineStr">
         <is>
           <t>■ 미수행 — 자원·현장 조건이 갖춰져야 할 수 있다. 함께 실어 「전부 확인했다」로 읽히지 않게 한다.</t>
         </is>
       </c>
     </row>
-    <row r="170">
-      <c r="A170" s="15" t="inlineStr">
+    <row r="181">
+      <c r="A181" s="15" t="inlineStr">
         <is>
           <t>TC-DP-01</t>
         </is>
       </c>
-      <c r="B170" s="15" t="inlineStr">
+      <c r="B181" s="15" t="inlineStr">
         <is>
           <t>정산</t>
         </is>
       </c>
-      <c r="C170" s="16" t="inlineStr">
+      <c r="C181" s="16" t="inlineStr">
         <is>
           <t>한 달을 실제로 정산해 입금·환급까지 마칠 수 있는가?</t>
         </is>
       </c>
-      <c r="D170" s="16" t="inlineStr">
+      <c r="D181" s="16" t="inlineStr">
         <is>
           <t>한 달 운영 후 실제 정산 1회전 수행</t>
         </is>
       </c>
-      <c r="E170" s="17" t="inlineStr">
+      <c r="E181" s="17" t="inlineStr">
         <is>
           <t>미수행</t>
         </is>
       </c>
-      <c r="F170" s="15" t="inlineStr"/>
-      <c r="G170" s="15" t="inlineStr"/>
-      <c r="H170" s="16" t="inlineStr">
+      <c r="F181" s="15" t="inlineStr"/>
+      <c r="G181" s="15" t="inlineStr"/>
+      <c r="H181" s="16" t="inlineStr">
         <is>
           <t>운영 데이터가 쌓여야 한다 — 사용자가 직접 해 보고 알려 주기로 함(2026-08-24)</t>
         </is>
       </c>
-      <c r="I170" s="16" t="inlineStr"/>
-    </row>
-    <row r="171">
-      <c r="A171" s="15" t="inlineStr">
+      <c r="I181" s="16" t="inlineStr"/>
+    </row>
+    <row r="182">
+      <c r="A182" s="15" t="inlineStr">
         <is>
           <t>TC-DP-02</t>
         </is>
       </c>
-      <c r="B171" s="15" t="inlineStr">
+      <c r="B182" s="15" t="inlineStr">
         <is>
           <t>메일</t>
         </is>
       </c>
-      <c r="C171" s="16" t="inlineStr">
+      <c r="C182" s="16" t="inlineStr">
         <is>
           <t>각자 실제 앱 비밀번호로 등록해 본인 주소에서 메일이 나가는가?</t>
         </is>
       </c>
-      <c r="D171" s="16" t="inlineStr">
+      <c r="D182" s="16" t="inlineStr">
         <is>
           <t>직원 7명이 각자 다음 메일에서 앱 비밀번호를 발급받아 등록</t>
         </is>
       </c>
-      <c r="E171" s="17" t="inlineStr">
+      <c r="E182" s="17" t="inlineStr">
         <is>
           <t>미수행</t>
         </is>
       </c>
-      <c r="F171" s="15" t="inlineStr"/>
-      <c r="G171" s="15" t="inlineStr"/>
-      <c r="H171" s="16" t="inlineStr"/>
-      <c r="I171" s="16" t="inlineStr">
+      <c r="F182" s="15" t="inlineStr"/>
+      <c r="G182" s="15" t="inlineStr"/>
+      <c r="H182" s="16" t="inlineStr"/>
+      <c r="I182" s="16" t="inlineStr">
         <is>
           <t>비밀번호는 본인만 다룰 수 있어 대신 확인할 수 없다</t>
         </is>
       </c>
     </row>
-    <row r="172">
-      <c r="A172" s="15" t="inlineStr">
+    <row r="183">
+      <c r="A183" s="15" t="inlineStr">
         <is>
           <t>TC-DP-03</t>
         </is>
       </c>
-      <c r="B172" s="15" t="inlineStr">
+      <c r="B183" s="15" t="inlineStr">
         <is>
           <t>휴가</t>
         </is>
       </c>
-      <c r="C172" s="16" t="inlineStr">
+      <c r="C183" s="16" t="inlineStr">
         <is>
           <t>실제 휴가를 신청·승인해 양쪽 메일이 도착하는가?</t>
         </is>
       </c>
-      <c r="D172" s="16" t="inlineStr">
+      <c r="D183" s="16" t="inlineStr">
         <is>
           <t>직원이 신청하고 대표이사가 승인 — 두 통 모두 수신 확인</t>
         </is>
       </c>
-      <c r="E172" s="17" t="inlineStr">
+      <c r="E183" s="17" t="inlineStr">
         <is>
           <t>미수행</t>
         </is>
       </c>
-      <c r="F172" s="15" t="inlineStr"/>
-      <c r="G172" s="15" t="inlineStr"/>
-      <c r="H172" s="16" t="inlineStr"/>
-      <c r="I172" s="16" t="inlineStr">
+      <c r="F183" s="15" t="inlineStr"/>
+      <c r="G183" s="15" t="inlineStr"/>
+      <c r="H183" s="16" t="inlineStr"/>
+      <c r="I183" s="16" t="inlineStr">
         <is>
           <t>승인 권한자가 직접 해야 한다</t>
         </is>
       </c>
     </row>
-    <row r="173">
-      <c r="A173" s="15" t="inlineStr">
+    <row r="184">
+      <c r="A184" s="15" t="inlineStr">
         <is>
           <t>TC-DP-04</t>
         </is>
       </c>
-      <c r="B173" s="15" t="inlineStr">
+      <c r="B184" s="15" t="inlineStr">
         <is>
           <t>휴가</t>
         </is>
       </c>
-      <c r="C173" s="16" t="inlineStr">
+      <c r="C184" s="16" t="inlineStr">
         <is>
           <t>공가를 쓰면 연차 잔여가 그대로인가?</t>
         </is>
       </c>
-      <c r="D173" s="16" t="inlineStr">
+      <c r="D184" s="16" t="inlineStr">
         <is>
           <t>공가를 실제로 등록한 뒤 연차 요약의 사용·잔여 확인</t>
         </is>
       </c>
-      <c r="E173" s="17" t="inlineStr">
+      <c r="E184" s="17" t="inlineStr">
         <is>
           <t>미수행</t>
         </is>
       </c>
-      <c r="F173" s="15" t="inlineStr"/>
-      <c r="G173" s="15" t="inlineStr"/>
-      <c r="H173" s="16" t="inlineStr">
+      <c r="F184" s="15" t="inlineStr"/>
+      <c r="G184" s="15" t="inlineStr"/>
+      <c r="H184" s="16" t="inlineStr">
         <is>
           <t>운영에 공가 기록이 아직 없다 — 처음 쓰실 때 함께 확인</t>
         </is>
       </c>
-      <c r="I173" s="16" t="inlineStr"/>
-    </row>
-    <row r="174">
-      <c r="A174" s="15" t="inlineStr">
+      <c r="I184" s="16" t="inlineStr"/>
+    </row>
+    <row r="185">
+      <c r="A185" s="15" t="inlineStr">
         <is>
           <t>TC-DP-05</t>
         </is>
       </c>
-      <c r="B174" s="15" t="inlineStr">
+      <c r="B185" s="15" t="inlineStr">
         <is>
           <t>안건</t>
         </is>
       </c>
-      <c r="C174" s="16" t="inlineStr">
+      <c r="C185" s="16" t="inlineStr">
         <is>
           <t>Jira 로 올릴 때 제목 뒤에 «_보고자» 가 붙는가?</t>
         </is>
       </c>
-      <c r="D174" s="16" t="inlineStr">
+      <c r="D185" s="16" t="inlineStr">
         <is>
           <t>보고자를 넣은 안건을 Jira 로 올려 제목 확인</t>
         </is>
       </c>
-      <c r="E174" s="17" t="inlineStr">
+      <c r="E185" s="17" t="inlineStr">
         <is>
           <t>미수행</t>
         </is>
       </c>
-      <c r="F174" s="15" t="inlineStr"/>
-      <c r="G174" s="15" t="inlineStr"/>
-      <c r="H174" s="16" t="inlineStr">
+      <c r="F185" s="15" t="inlineStr"/>
+      <c r="G185" s="15" t="inlineStr"/>
+      <c r="H185" s="16" t="inlineStr">
         <is>
           <t>실제 Jira 이슈가 만들어지므로 시험용으로 올리지 않았다</t>
         </is>
       </c>
-      <c r="I174" s="16" t="inlineStr">
+      <c r="I185" s="16" t="inlineStr">
         <is>
           <t>여러 번 올려도 겹쳐 붙지 않아야 한다</t>
         </is>
       </c>
     </row>
-    <row r="175">
-      <c r="A175" s="15" t="inlineStr">
+    <row r="186">
+      <c r="A186" s="15" t="inlineStr">
         <is>
           <t>TC-DP-06</t>
         </is>
       </c>
-      <c r="B175" s="15" t="inlineStr">
+      <c r="B186" s="15" t="inlineStr">
         <is>
           <t>회의록</t>
         </is>
       </c>
-      <c r="C175" s="16" t="inlineStr">
+      <c r="C186" s="16" t="inlineStr">
         <is>
           <t>여러 사람이 «동시에» 자기 칸을 적어도 부딪히지 않는가?</t>
         </is>
       </c>
-      <c r="D175" s="16" t="inlineStr">
+      <c r="D186" s="16" t="inlineStr">
         <is>
           <t>두 사람이 같은 회의록을 동시에 열고 각자 저장</t>
         </is>
       </c>
-      <c r="E175" s="17" t="inlineStr">
+      <c r="E186" s="17" t="inlineStr">
         <is>
           <t>미수행</t>
         </is>
       </c>
-      <c r="F175" s="15" t="inlineStr"/>
-      <c r="G175" s="15" t="inlineStr"/>
-      <c r="H175" s="16" t="inlineStr">
+      <c r="F186" s="15" t="inlineStr"/>
+      <c r="G186" s="15" t="inlineStr"/>
+      <c r="H186" s="16" t="inlineStr">
         <is>
           <t>사람이 둘 이상 있어야 한다 — 실제 회의에서 확인</t>
         </is>
       </c>
-      <c r="I175" s="16" t="inlineStr">
+      <c r="I186" s="16" t="inlineStr">
         <is>
           <t>칸을 나눈 것이 이 문제를 없애기 위한 설계다</t>
         </is>
       </c>
     </row>
-    <row r="176">
-      <c r="A176" s="15" t="inlineStr">
+    <row r="187">
+      <c r="A187" s="15" t="inlineStr">
         <is>
           <t>TC-DP-07</t>
         </is>
       </c>
-      <c r="B176" s="15" t="inlineStr">
+      <c r="B187" s="15" t="inlineStr">
         <is>
           <t>하이패스</t>
         </is>
       </c>
-      <c r="C176" s="16" t="inlineStr">
+      <c r="C187" s="16" t="inlineStr">
         <is>
           <t>건별 하이패스 메일이 직원에게 도착하는가?</t>
         </is>
       </c>
-      <c r="D176" s="16" t="inlineStr">
+      <c r="D187" s="16" t="inlineStr">
         <is>
           <t>「메일 보내기」를 눌러 실제 수신 확인</t>
         </is>
       </c>
-      <c r="E176" s="17" t="inlineStr">
+      <c r="E187" s="17" t="inlineStr">
         <is>
           <t>미수행</t>
         </is>
       </c>
-      <c r="F176" s="15" t="inlineStr"/>
-      <c r="G176" s="15" t="inlineStr"/>
-      <c r="H176" s="16" t="inlineStr">
+      <c r="F187" s="15" t="inlineStr"/>
+      <c r="G187" s="15" t="inlineStr"/>
+      <c r="H187" s="16" t="inlineStr">
         <is>
           <t>실제 직원에게 나가므로 승인 전까지 누르지 않았다</t>
         </is>
       </c>
-      <c r="I176" s="16" t="inlineStr"/>
-    </row>
-    <row r="177">
-      <c r="A177" s="15" t="inlineStr">
+      <c r="I187" s="16" t="inlineStr"/>
+    </row>
+    <row r="188">
+      <c r="A188" s="15" t="inlineStr">
         <is>
           <t>TC-DP-08</t>
         </is>
       </c>
-      <c r="B177" s="15" t="inlineStr">
+      <c r="B188" s="15" t="inlineStr">
         <is>
           <t>일정</t>
         </is>
       </c>
-      <c r="C177" s="16" t="inlineStr">
+      <c r="C188" s="16" t="inlineStr">
         <is>
           <t>네이버 길찾기 링크가 실제로 열리는가?</t>
         </is>
       </c>
-      <c r="D177" s="16" t="inlineStr">
+      <c r="D188" s="16" t="inlineStr">
         <is>
           <t>「이동」 일정에서 링크를 눌러 길찾기 화면 확인</t>
         </is>
       </c>
-      <c r="E177" s="17" t="inlineStr">
+      <c r="E188" s="17" t="inlineStr">
         <is>
           <t>미수행</t>
         </is>
       </c>
-      <c r="F177" s="15" t="inlineStr"/>
-      <c r="G177" s="15" t="inlineStr"/>
-      <c r="H177" s="16" t="inlineStr">
+      <c r="F188" s="15" t="inlineStr"/>
+      <c r="G188" s="15" t="inlineStr"/>
+      <c r="H188" s="16" t="inlineStr">
         <is>
           <t>브라우저 패널이 map.naver.com 을 «정책으로» 막는다 — 2026-09-12 에 다시 시도해도 같았다</t>
         </is>
       </c>
-      <c r="I177" s="16" t="inlineStr">
+      <c r="I188" s="16" t="inlineStr">
         <is>
           <t>일반 브라우저에서 눌러 확인해야 한다</t>
         </is>
@@ -8276,11 +8749,11 @@
     </row>
   </sheetData>
   <mergeCells count="2">
-    <mergeCell ref="A169:I169"/>
+    <mergeCell ref="A180:I180"/>
     <mergeCell ref="A2:I2"/>
   </mergeCells>
   <dataValidations count="1">
-    <dataValidation sqref="E2:E177" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="E2:E188" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"적합,부적합,미수행"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>